<commit_message>
feat: job history for employees for easier unit transfer
</commit_message>
<xml_diff>
--- a/TimeManager.Backend/wwwroot/assets/timemanager_jobprofile_bulk_import_example.xlsx
+++ b/TimeManager.Backend/wwwroot/assets/timemanager_jobprofile_bulk_import_example.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agarbuja1s\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\agarbuja1s\source\repos\TimeManager\TimeManager.Backend\wwwroot\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEFBE0DD-06AE-4870-8860-802604838B85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9A95703-8ACF-42DE-946A-C32AA2C9F864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{F5256E3E-E473-4FB4-9FCA-8052D07D2AAC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Role</t>
   </si>
@@ -51,6 +51,12 @@
   </si>
   <si>
     <t>Index</t>
+  </si>
+  <si>
+    <t>Hire Date</t>
+  </si>
+  <si>
+    <t>MM/DD/YYYY</t>
   </si>
 </sst>
 </file>
@@ -455,15 +461,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{523E7C17-75F0-4D89-9D19-2E6E884DE609}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="70.7109375" customWidth="1"/>
+    <col min="4" max="4" width="24.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -473,8 +480,11 @@
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>123455</v>
       </c>
@@ -483,6 +493,9 @@
       </c>
       <c r="C2" t="s">
         <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>